<commit_message>
Add batch processing with Excel saved after each batch
</commit_message>
<xml_diff>
--- a/acnc_charities_sample.xlsx
+++ b/acnc_charities_sample.xlsx
@@ -425,10 +425,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="59" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -1094,6 +1094,1541 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>East Gippsland Verge Gardens and Landcare Inc.</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12189591217</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>egvergegardens@outlook.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Southern Tablelands Open Gardens Association Incorporated</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>64114537881</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>info@stoga.org.au</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Greenough Museum &amp; Gardens Community Association Inc.</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>84294031040</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>treasurer@greenoughmuseum.org.au</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>THE TRUSTEE FOR FOUNDATION AND FRIENDS OF THE BOTANIC GARDENS TRUST</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>50837658196</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Foundation.friends@rbgsyd.nsw.gov.au</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Australian Association of Friends of Botanic Gardens Inc</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>99467025064</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>jill@creativedialogue.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Camelot Community Garden</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>53155807041</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>camelotcommunitygarden@gmail.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Ocean Gardens Inc</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>94429163573</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>reception@oceangardens.com.au</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Leederville Gardens Inc</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>63094298628</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>secretary@leedervillegardens.com.au</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Busselton Community Garden</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>42937465518</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>busseltoncommunitygardens@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Friends Of Gardens And Parks</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>34986776565</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GeorgeNelsonAU@gmail.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ultimo Community Garden</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>95880616252</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>trevorclarkson@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>OPERA IN THE GARDENS INC</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>15842912650</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>goondiwindiopera@gmail.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Topsoil Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>82376282275</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>admin@topsoilgarden.org</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Orana Gardens Ltd</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>98081776687</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>clintg@oranagardens.com.au</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>THE GARDEN MELBOURNE LIMITED</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>86635867248</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>info@thefield.church</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>The Trustee for Foundation and Friends of the Botanic Gardens Charitable Fund</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>92871129496</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>foundation.friends@rbgsyd.nsw.gov.au</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>The Leura Gardens Festival Incorporated</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>36635596991</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>zentricity53@gmail.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Lucas Gardens School P&amp;C</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>62745594304</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>secretary.lucasgardens.pc@google.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Anglican Parish Of Bulahdelah/Tea Gardens</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>78883692372</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>office@parishbtgk.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Bayside Garden Club Inc</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>48982739291</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>baysidegc01@gmail.com.au</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>The Anglican Parish Of Toorak Gardens</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>85943986012</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>governance@adelaideanglicans.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SIDRAH GARDENS SCHOOL LIMITED</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>18634025737</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>munirabdul86@gmail.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>The Anglican Parish of Clarence Gardens</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>16261421699</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>governance@adelaideanglicans.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Church Of Christ Hampstead Gardens</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>47806369292</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>office@hampsteadgardenscofc.org.au</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Geelong Organic Gardeners Inc</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>19714390961</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>gog.geelong@gmail.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Cherry Gardens Uniting Church</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>44249955417</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>cherrychurchinfo@gmail.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>THE HOE GARDEN FOUNDATION LIMITED</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>42697424141</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>hoegardenfoundation@gmail.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Brompton Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>60277040528</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>communitygardenbrompton@gmail.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Tea Gardens Baptist Church</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>55372497882</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>secretary@teagardensbaptist.org.au</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Australian Garden Council  Limited</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>67614881677</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>info@gardencouncil.org</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Botanica Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>59471794828</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>botanicacommunitygarden@gmail.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Warrnambool Community Garden Inc.</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>32710842442</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>admin@wcg3280.org.au</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Padbury Community Garden Inc.</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>73906670127</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>padburycommunitygarden@gmail.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Callala Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>87342085609</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Callalacommunitygarden@gmail.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Banksia Gardens Association Inc</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>54264568661</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>admin@banksiagardens.org.au</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Thalassa Park and Gardens Trust</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>85237093573</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>normanville32@bigpond.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Royal Tasmanian Botanical Gardens</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>75542604274</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>contact@gardens.tas.gov.au</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>WILDFLOWER, GARDENS FOR GOOD LIMITED</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>98742903078</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>roman@wildflower.org.au</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Maroubra Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>70254639936</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Gargarro Botanic Garden Ltd</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>63610887986</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>michael.watt@msgroup.net.au</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Kariong Eco Garden Inc</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>13852216759</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>pfa.farina@gmail.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Doncaster Community Gardeners Incorporated</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>44236214226</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>TREVOREDDY@OPTUSNET.COM.AU</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Pinjarra Community Garden Inc</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>38272873276</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>info@pinjarracommunitygarden.com.au</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>TASMANIAN BUSHLAND GARDEN INCORPORATED</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>66773941212</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>vexternest@gmx.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>EMILY'S GARDEN FOUNDATION LTD</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>16687969428</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>cherylmckenna79@icloud.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Foley Gardens Retirement Village</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>21007332174</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>agedcare@sydneycatholic.org</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Frederick Miller Community Garden</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>61998274313</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>stevebelton5@gmail.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MOSSMAN BOTANIC GARDEN LTD</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>36635423068</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ceo@mossmanbotanicgarden.com.au</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>VETERANS ORGANIC GARDEN LIMITED</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>21662369735</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>davidgowerfreeman@icloud.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>FRIENDS OF MCMAUGH GARDENS INC</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>72527765606</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>friendsofmcmaughs@gmail.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Punt Hill Community Garden</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>52606799397</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>punthillcomgarden@gmail.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Easy Care Gardening Inc</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>96338250354</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>info@easycaregardening.org.au</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Chilwell Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>79383997927</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>chilwellcommunitygarden@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Canterbury Gardens Community Church</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>80201841076</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>accounts@cgcc.org.au</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Portland Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>35282136568</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>pcg.treasurer@outlook.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Armidale Botanic Garden Inc</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>65180016952</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Nedgardendesign@outlook.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>National Rock Garden Trust</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>41345443328</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>info@gsa.org.au</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Thrive Community Garden Inc</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>94806597496</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>woody@thrivecommunitygarden.org</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Globalscope Brisbane: The Garden Ltd</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>95621808464</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>doctorschlipf@gmail.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Jimboomba Community Garden Inc</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>34462783925</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>secretary.jcg@gmail.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Global Gardens of Peace Incorporated</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>44362890385</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>secretary@globalgardensofpeace.org</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Mulwala Community Garden Incorporated</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>33758804868</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>mulwalacommunitygarden@gmail.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Hurstville Community Garden Association</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>54757279533</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>hurstvillecga@gmail.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Olive Pink Botanic Garden</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>94163536423</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>curator@opbg.com.au</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>BUDERIM GARDEN CLUB INCORPORATED</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>70509008891</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>john.lyon1@bigpond.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Open Gardens Canberra Inc</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>80136609319</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>maindav@bigpond.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Kwinana Community Gardens Incorporated</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>96336810368</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>secretary@kwinanacommunitygardens.org</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>GOONDIWINDI BOTANIC GARDENS INC</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>83823810450</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>goondiwindibotanicgardens@gmail.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Sustainable Gardening Australia Foundation</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>47508099142</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>p.howey@sgaonline.org.au</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>COMMUNITY GARDENS AUSTRALIA LIMITED</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>88666023034</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>info@communitygarden.org.au</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>